<commit_message>
verse comparison list: drop Leviticus 6:25 row (matches the JSON data)
Source xlsx now in sync with data/verseComparisonList.json +
verseComparisons.json, which already had it removed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/500_verse_comparison_list.xlsx
+++ b/500_verse_comparison_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\claude\bible-translation-guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD93A00D-2712-4B9C-96B7-4E09BE3A4D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E59B025-94C0-40B5-9D09-7498B0BA9C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D265D67B-1933-4DB5-8411-0C36F9C5B8B1}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1483" uniqueCount="558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="557">
   <si>
     <t>Reference</t>
   </si>
@@ -1477,9 +1477,6 @@
   </si>
   <si>
     <t>1 Timothy 1:10</t>
-  </si>
-  <si>
-    <t>Leviticus 6:25</t>
   </si>
   <si>
     <t>Matthew 4:24</t>
@@ -2559,7 +2556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57C3E312-5580-46BC-BC59-D9E2C6392FA6}">
-  <dimension ref="A1:D503"/>
+  <dimension ref="A1:D502"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
@@ -6500,490 +6497,490 @@
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
+        <v>494</v>
+      </c>
+      <c r="B358" t="s">
         <v>495</v>
-      </c>
-      <c r="B358" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B359" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B360" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B361" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B362" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B363" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B364" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B365" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B366" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B367" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B368" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="369" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="B369" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="370" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B370" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="371" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A371" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B371" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="372" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B372" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="373" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B373" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="374" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B374" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="375" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A375" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B375" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="376" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B376" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="377" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B377" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="378" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B378" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="379" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B379" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="380" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B380" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="381" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B381" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="382" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B382" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="383" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B383" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="384" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B384" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="385" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B385" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="386" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B386" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="387" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B387" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="388" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="B388" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="389" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B389" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="390" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="B390" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="391" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A391" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B391" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="392" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B392" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="393" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B393" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="394" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B394" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="395" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B395" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="396" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B396" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="397" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B397" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="398" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B398" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="399" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B399" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="400" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B400" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="401" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B401" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="402" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B402" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="403" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B403" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="404" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B404" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="405" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B405" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="406" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B406" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="407" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B407" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="408" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A408" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B408" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="409" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B409" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="410" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B410" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="411" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B411" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="412" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B412" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="413" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B413" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="414" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B414" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="415" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B415" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="416" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B416" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B417" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B418" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.35">
@@ -7088,7 +7085,7 @@
         <v>403</v>
       </c>
       <c r="D427" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.35">
@@ -7102,7 +7099,7 @@
         <v>403</v>
       </c>
       <c r="D428" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.35">
@@ -7116,7 +7113,7 @@
         <v>403</v>
       </c>
       <c r="D429" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.35">
@@ -7130,7 +7127,7 @@
         <v>403</v>
       </c>
       <c r="D430" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.35">
@@ -7144,7 +7141,7 @@
         <v>403</v>
       </c>
       <c r="D431" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.35">
@@ -7158,7 +7155,7 @@
         <v>403</v>
       </c>
       <c r="D432" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.35">
@@ -7172,7 +7169,7 @@
         <v>403</v>
       </c>
       <c r="D433" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.35">
@@ -7186,7 +7183,7 @@
         <v>403</v>
       </c>
       <c r="D434" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.35">
@@ -7200,7 +7197,7 @@
         <v>403</v>
       </c>
       <c r="D435" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.35">
@@ -7214,7 +7211,7 @@
         <v>403</v>
       </c>
       <c r="D436" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.35">
@@ -7228,7 +7225,7 @@
         <v>403</v>
       </c>
       <c r="D437" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.35">
@@ -7242,7 +7239,7 @@
         <v>403</v>
       </c>
       <c r="D438" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.35">
@@ -7580,18 +7577,18 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
-        <v>485</v>
+        <v>435</v>
       </c>
       <c r="B466" t="s">
         <v>64</v>
       </c>
       <c r="C466" t="s">
-        <v>480</v>
+        <v>436</v>
       </c>
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B467" t="s">
         <v>64</v>
@@ -7602,7 +7599,7 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B468" t="s">
         <v>64</v>
@@ -7613,7 +7610,7 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B469" t="s">
         <v>64</v>
@@ -7624,7 +7621,7 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B470" t="s">
         <v>64</v>
@@ -7635,7 +7632,7 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B471" t="s">
         <v>64</v>
@@ -7646,7 +7643,7 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
-        <v>441</v>
+        <v>476</v>
       </c>
       <c r="B472" t="s">
         <v>64</v>
@@ -7657,18 +7654,21 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
-        <v>476</v>
+        <v>467</v>
       </c>
       <c r="B473" t="s">
         <v>64</v>
       </c>
       <c r="C473" t="s">
-        <v>436</v>
+        <v>65</v>
+      </c>
+      <c r="D473" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B474" t="s">
         <v>64</v>
@@ -7682,7 +7682,7 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
-        <v>469</v>
+        <v>431</v>
       </c>
       <c r="B475" t="s">
         <v>64</v>
@@ -7691,12 +7691,12 @@
         <v>65</v>
       </c>
       <c r="D475" t="s">
-        <v>468</v>
+        <v>432</v>
       </c>
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B476" t="s">
         <v>64</v>
@@ -7710,7 +7710,7 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="B477" t="s">
         <v>64</v>
@@ -7719,12 +7719,12 @@
         <v>65</v>
       </c>
       <c r="D477" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A478" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B478" t="s">
         <v>64</v>
@@ -7738,7 +7738,7 @@
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
-        <v>430</v>
+        <v>455</v>
       </c>
       <c r="B479" t="s">
         <v>64</v>
@@ -7747,12 +7747,12 @@
         <v>65</v>
       </c>
       <c r="D479" t="s">
-        <v>429</v>
+        <v>456</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B480" t="s">
         <v>64</v>
@@ -7766,7 +7766,7 @@
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A481" t="s">
-        <v>457</v>
+        <v>63</v>
       </c>
       <c r="B481" t="s">
         <v>64</v>
@@ -7775,12 +7775,12 @@
         <v>65</v>
       </c>
       <c r="D481" t="s">
-        <v>456</v>
+        <v>59</v>
       </c>
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A482" t="s">
-        <v>63</v>
+        <v>454</v>
       </c>
       <c r="B482" t="s">
         <v>64</v>
@@ -7788,13 +7788,10 @@
       <c r="C482" t="s">
         <v>65</v>
       </c>
-      <c r="D482" t="s">
-        <v>59</v>
-      </c>
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A483" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="B483" t="s">
         <v>64</v>
@@ -7805,7 +7802,7 @@
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A484" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B484" t="s">
         <v>64</v>
@@ -7816,7 +7813,7 @@
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A485" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="B485" t="s">
         <v>64</v>
@@ -7827,7 +7824,7 @@
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A486" t="s">
-        <v>470</v>
+        <v>492</v>
       </c>
       <c r="B486" t="s">
         <v>64</v>
@@ -7849,18 +7846,18 @@
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A488" t="s">
-        <v>494</v>
+        <v>443</v>
       </c>
       <c r="B488" t="s">
         <v>64</v>
       </c>
       <c r="C488" t="s">
-        <v>65</v>
+        <v>444</v>
       </c>
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A489" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B489" t="s">
         <v>64</v>
@@ -7871,7 +7868,7 @@
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A490" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B490" t="s">
         <v>64</v>
@@ -7882,7 +7879,7 @@
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A491" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B491" t="s">
         <v>64</v>
@@ -7893,7 +7890,7 @@
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A492" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B492" t="s">
         <v>64</v>
@@ -7904,7 +7901,7 @@
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A493" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B493" t="s">
         <v>64</v>
@@ -7915,7 +7912,7 @@
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A494" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="B494" t="s">
         <v>64</v>
@@ -7926,7 +7923,7 @@
     </row>
     <row r="495" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A495" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="B495" t="s">
         <v>64</v>
@@ -7937,7 +7934,7 @@
     </row>
     <row r="496" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A496" t="s">
-        <v>466</v>
+        <v>485</v>
       </c>
       <c r="B496" t="s">
         <v>64</v>
@@ -8012,22 +8009,11 @@
         <v>444</v>
       </c>
     </row>
-    <row r="503" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A503" t="s">
-        <v>492</v>
-      </c>
-      <c r="B503" t="s">
-        <v>64</v>
-      </c>
-      <c r="C503" t="s">
-        <v>444</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D504">
-    <sortCondition ref="B2:B504"/>
-    <sortCondition ref="C2:C504"/>
-    <sortCondition ref="D2:D504"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D503">
+    <sortCondition ref="B2:B503"/>
+    <sortCondition ref="C2:C503"/>
+    <sortCondition ref="D2:D503"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>